<commit_message>
data(pricing): promote audited to canonical; archive pre-audit snapshot
CEO authority per chat: audited Excel passed expert + auditor judgment, lifts
all justified by net-margin math, healthy SKUs preserved, math hygiene cleaned.

- master-pricing-2026-05-01-snapshot.xlsx ← audited file (now canonical)
- master-pricing-2026-04-archived-pre-audit.xlsx ← original pre-audit (preserved
  for reference)
- master-pricing-2026-05-01-audited.xlsx ← removed (was transitional output)

The canonical Excel is now the source of truth for:
- GHL custom fields (T1/T2/T3 quote tiers)
- Quote drafting workflows (Phase 2)
- AI Quote Drafter (Phase 6.1)
- Sub rate schedule (Sub Labour column)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pricing/master-pricing-2026-05-01-snapshot.xlsx
+++ b/data/pricing/master-pricing-2026-05-01-snapshot.xlsx
@@ -4242,19 +4242,19 @@
         <v>191</v>
       </c>
       <c r="M5" s="138" t="n">
-        <v>530</v>
+        <v>800</v>
       </c>
       <c r="N5" s="138" t="n">
-        <v>420</v>
+        <v>630</v>
       </c>
       <c r="O5" s="138" t="n">
-        <v>320</v>
+        <v>480</v>
       </c>
       <c r="P5" s="139" t="n">
-        <v>191</v>
+        <v>381.7272727272726</v>
       </c>
       <c r="Q5" s="140" t="n">
-        <v>0.499761904761905</v>
+        <v>0.6665079365079365</v>
       </c>
       <c r="R5" s="137" t="inlineStr">
         <is>
@@ -4316,19 +4316,19 @@
         <v>143</v>
       </c>
       <c r="M6" s="138" t="n">
-        <v>390</v>
+        <v>680</v>
       </c>
       <c r="N6" s="138" t="n">
-        <v>310</v>
+        <v>540</v>
       </c>
       <c r="O6" s="138" t="n">
-        <v>250</v>
+        <v>440</v>
       </c>
       <c r="P6" s="139" t="n">
-        <v>139</v>
+        <v>347.9090909090909</v>
       </c>
       <c r="Q6" s="140" t="n">
-        <v>0.49258064516129</v>
+        <v>0.7087037037037037</v>
       </c>
       <c r="R6" s="137" t="inlineStr">
         <is>
@@ -4390,19 +4390,19 @@
         <v>261</v>
       </c>
       <c r="M7" s="138" t="n">
-        <v>780</v>
+        <v>1000</v>
       </c>
       <c r="N7" s="138" t="n">
-        <v>600</v>
+        <v>770</v>
       </c>
       <c r="O7" s="138" t="n">
-        <v>490</v>
+        <v>630</v>
       </c>
       <c r="P7" s="139" t="n">
-        <v>284</v>
+        <v>439</v>
       </c>
       <c r="Q7" s="140" t="n">
-        <v>0.5215</v>
+        <v>0.6271428571428571</v>
       </c>
       <c r="R7" s="137" t="inlineStr">
         <is>
@@ -4473,10 +4473,10 @@
         <v>550</v>
       </c>
       <c r="P8" s="139" t="n">
-        <v>321</v>
+        <v>321.2727272727273</v>
       </c>
       <c r="Q8" s="140" t="n">
-        <v>0.512173913043478</v>
+        <v>0.5121739130434783</v>
       </c>
       <c r="R8" s="137" t="inlineStr">
         <is>
@@ -4538,19 +4538,19 @@
         <v>128</v>
       </c>
       <c r="M9" s="138" t="n">
-        <v>330</v>
+        <v>620</v>
       </c>
       <c r="N9" s="138" t="n">
-        <v>270</v>
+        <v>510</v>
       </c>
       <c r="O9" s="138" t="n">
-        <v>210</v>
+        <v>400</v>
       </c>
       <c r="P9" s="139" t="n">
-        <v>117</v>
+        <v>335.6363636363636</v>
       </c>
       <c r="Q9" s="140" t="n">
-        <v>0.478518518518519</v>
+        <v>0.7239215686274509</v>
       </c>
       <c r="R9" s="137" t="inlineStr">
         <is>
@@ -4621,10 +4621,10 @@
         <v>420</v>
       </c>
       <c r="P10" s="139" t="n">
-        <v>287</v>
+        <v>286.8181818181818</v>
       </c>
       <c r="Q10" s="145" t="n">
-        <v>0.595283018867925</v>
+        <v>0.5952830188679245</v>
       </c>
       <c r="R10" s="143" t="inlineStr">
         <is>
@@ -4680,10 +4680,10 @@
         <v>3</v>
       </c>
       <c r="K11" s="144" t="n">
-        <v>220</v>
+        <v>199.5</v>
       </c>
       <c r="L11" s="144" t="n">
-        <v>271</v>
+        <v>250.5</v>
       </c>
       <c r="M11" s="144" t="n">
         <v>860</v>
@@ -4695,10 +4695,10 @@
         <v>550</v>
       </c>
       <c r="P11" s="139" t="n">
-        <v>376</v>
+        <v>376.7727272727273</v>
       </c>
       <c r="Q11" s="145" t="n">
-        <v>0.599855072463768</v>
+        <v>0.6006521739130435</v>
       </c>
       <c r="R11" s="143" t="inlineStr">
         <is>
@@ -4754,10 +4754,10 @@
         <v>3</v>
       </c>
       <c r="K12" s="144" t="n">
-        <v>285</v>
+        <v>261</v>
       </c>
       <c r="L12" s="144" t="n">
-        <v>343</v>
+        <v>319</v>
       </c>
       <c r="M12" s="144" t="n">
         <v>1050</v>
@@ -4769,10 +4769,10 @@
         <v>690</v>
       </c>
       <c r="P12" s="147" t="n">
-        <v>464</v>
+        <v>462.8181818181818</v>
       </c>
       <c r="Q12" s="145" t="n">
-        <v>0.593255813953488</v>
+        <v>0.5919767441860465</v>
       </c>
       <c r="R12" s="143" t="inlineStr">
         <is>
@@ -4828,10 +4828,10 @@
         <v>3</v>
       </c>
       <c r="K13" s="144" t="n">
-        <v>350</v>
+        <v>319</v>
       </c>
       <c r="L13" s="144" t="n">
-        <v>418</v>
+        <v>387</v>
       </c>
       <c r="M13" s="144" t="n">
         <v>1320</v>
@@ -4843,10 +4843,10 @@
         <v>860</v>
       </c>
       <c r="P13" s="147" t="n">
-        <v>567</v>
+        <v>567.5454545454545</v>
       </c>
       <c r="Q13" s="145" t="n">
-        <v>0.59352380952381</v>
+        <v>0.5945714285714285</v>
       </c>
       <c r="R13" s="143" t="inlineStr">
         <is>
@@ -4902,10 +4902,10 @@
         <v>40</v>
       </c>
       <c r="K14" s="144" t="n">
-        <v>310</v>
+        <v>310.5</v>
       </c>
       <c r="L14" s="144" t="n">
-        <v>429</v>
+        <v>429.5</v>
       </c>
       <c r="M14" s="144" t="n">
         <v>1320</v>
@@ -4917,10 +4917,10 @@
         <v>890</v>
       </c>
       <c r="P14" s="147" t="n">
-        <v>571</v>
+        <v>570.4999999999999</v>
       </c>
       <c r="Q14" s="145" t="n">
-        <v>0.571</v>
+        <v>0.5704999999999999</v>
       </c>
       <c r="R14" s="143" t="inlineStr">
         <is>
@@ -4991,10 +4991,10 @@
         <v>1080</v>
       </c>
       <c r="P15" s="147" t="n">
-        <v>738</v>
+        <v>737.5454545454545</v>
       </c>
       <c r="Q15" s="145" t="n">
-        <v>0.587898550724638</v>
+        <v>0.5878985507246377</v>
       </c>
       <c r="R15" s="143" t="inlineStr">
         <is>
@@ -5050,10 +5050,10 @@
         <v>55</v>
       </c>
       <c r="K16" s="144" t="n">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="L16" s="144" t="n">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="M16" s="144" t="n">
         <v>2150</v>
@@ -5065,10 +5065,10 @@
         <v>1320</v>
       </c>
       <c r="P16" s="148" t="n">
-        <v>851</v>
+        <v>849.090909090909</v>
       </c>
       <c r="Q16" s="145" t="n">
-        <v>0.563975903614458</v>
+        <v>0.5626506024096385</v>
       </c>
       <c r="R16" s="143" t="inlineStr">
         <is>
@@ -5139,10 +5139,10 @@
         <v>1660</v>
       </c>
       <c r="P17" s="148" t="n">
-        <v>1036</v>
+        <v>1035.545454545455</v>
       </c>
       <c r="Q17" s="145" t="n">
-        <v>0.558382352941176</v>
+        <v>0.5583823529411764</v>
       </c>
       <c r="R17" s="143" t="inlineStr">
         <is>
@@ -5198,10 +5198,10 @@
         <v>40</v>
       </c>
       <c r="K18" s="151" t="n">
-        <v>360</v>
+        <v>357.5</v>
       </c>
       <c r="L18" s="151" t="n">
-        <v>570</v>
+        <v>567.5</v>
       </c>
       <c r="M18" s="151" t="n">
         <v>1660</v>
@@ -5213,10 +5213,10 @@
         <v>1100</v>
       </c>
       <c r="P18" s="147" t="n">
-        <v>685</v>
+        <v>687.0454545454545</v>
       </c>
       <c r="Q18" s="140" t="n">
-        <v>0.545652173913043</v>
+        <v>0.5476449275362318</v>
       </c>
       <c r="R18" s="150" t="inlineStr">
         <is>
@@ -5272,10 +5272,10 @@
         <v>45</v>
       </c>
       <c r="K19" s="151" t="n">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="L19" s="151" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="M19" s="151" t="n">
         <v>2090</v>
@@ -5287,10 +5287,10 @@
         <v>1320</v>
       </c>
       <c r="P19" s="148" t="n">
-        <v>844</v>
+        <v>843.090909090909</v>
       </c>
       <c r="Q19" s="145" t="n">
-        <v>0.5593373493975899</v>
+        <v>0.5586746987951807</v>
       </c>
       <c r="R19" s="150" t="inlineStr">
         <is>
@@ -5346,10 +5346,10 @@
         <v>55</v>
       </c>
       <c r="K20" s="151" t="n">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="L20" s="151" t="n">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="M20" s="151" t="n">
         <v>2530</v>
@@ -5361,10 +5361,10 @@
         <v>1600</v>
       </c>
       <c r="P20" s="148" t="n">
-        <v>974</v>
+        <v>976.090909090909</v>
       </c>
       <c r="Q20" s="140" t="n">
-        <v>0.538442211055276</v>
+        <v>0.5395477386934673</v>
       </c>
       <c r="R20" s="150" t="inlineStr">
         <is>
@@ -5438,7 +5438,7 @@
         <v>1085</v>
       </c>
       <c r="Q21" s="140" t="n">
-        <v>0.5166666666666671</v>
+        <v>0.5166666666666667</v>
       </c>
       <c r="R21" s="150" t="inlineStr">
         <is>
@@ -5494,10 +5494,10 @@
         <v>43</v>
       </c>
       <c r="K22" s="144" t="n">
-        <v>370</v>
+        <v>368.5</v>
       </c>
       <c r="L22" s="144" t="n">
-        <v>527</v>
+        <v>525.5</v>
       </c>
       <c r="M22" s="144" t="n">
         <v>1600</v>
@@ -5509,10 +5509,10 @@
         <v>1050</v>
       </c>
       <c r="P22" s="147" t="n">
-        <v>628</v>
+        <v>629.0454545454545</v>
       </c>
       <c r="Q22" s="140" t="n">
-        <v>0.543543307086614</v>
+        <v>0.5448425196850394</v>
       </c>
       <c r="R22" s="143" t="inlineStr">
         <is>
@@ -5568,10 +5568,10 @@
         <v>48</v>
       </c>
       <c r="K23" s="144" t="n">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="L23" s="144" t="n">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="M23" s="144" t="n">
         <v>2040</v>
@@ -5583,10 +5583,10 @@
         <v>1320</v>
       </c>
       <c r="P23" s="148" t="n">
-        <v>884</v>
+        <v>882.090909090909</v>
       </c>
       <c r="Q23" s="145" t="n">
-        <v>0.585843373493976</v>
+        <v>0.5845180722891566</v>
       </c>
       <c r="R23" s="143" t="inlineStr">
         <is>
@@ -5642,10 +5642,10 @@
         <v>58</v>
       </c>
       <c r="K24" s="144" t="n">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="L24" s="144" t="n">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="M24" s="144" t="n">
         <v>2420</v>
@@ -5657,10 +5657,10 @@
         <v>1600</v>
       </c>
       <c r="P24" s="148" t="n">
-        <v>952</v>
+        <v>948.5454545454545</v>
       </c>
       <c r="Q24" s="140" t="n">
-        <v>0.542331606217617</v>
+        <v>0.5406217616580311</v>
       </c>
       <c r="R24" s="143" t="inlineStr">
         <is>
@@ -5734,7 +5734,7 @@
         <v>1406</v>
       </c>
       <c r="Q25" s="145" t="n">
-        <v>0.585833333333333</v>
+        <v>0.5858333333333333</v>
       </c>
       <c r="R25" s="143" t="inlineStr">
         <is>
@@ -5790,10 +5790,10 @@
         <v>43</v>
       </c>
       <c r="K26" s="151" t="n">
-        <v>410</v>
+        <v>409.5</v>
       </c>
       <c r="L26" s="151" t="n">
-        <v>658</v>
+        <v>657.5</v>
       </c>
       <c r="M26" s="151" t="n">
         <v>1820</v>
@@ -5805,10 +5805,10 @@
         <v>1210</v>
       </c>
       <c r="P26" s="147" t="n">
-        <v>697</v>
+        <v>697.0454545454545</v>
       </c>
       <c r="Q26" s="140" t="n">
-        <v>0.514228187919463</v>
+        <v>0.5145973154362415</v>
       </c>
       <c r="R26" s="150" t="inlineStr">
         <is>
@@ -5864,10 +5864,10 @@
         <v>48</v>
       </c>
       <c r="K27" s="151" t="n">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="L27" s="151" t="n">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="M27" s="151" t="n">
         <v>2310</v>
@@ -5879,10 +5879,10 @@
         <v>1550</v>
       </c>
       <c r="P27" s="148" t="n">
-        <v>956</v>
+        <v>958.090909090909</v>
       </c>
       <c r="Q27" s="145" t="n">
-        <v>0.559414893617021</v>
+        <v>0.5605851063829786</v>
       </c>
       <c r="R27" s="150" t="inlineStr">
         <is>
@@ -6012,10 +6012,10 @@
         <v>68</v>
       </c>
       <c r="K29" s="151" t="n">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="L29" s="151" t="n">
-        <v>1178</v>
+        <v>1181</v>
       </c>
       <c r="M29" s="151" t="n">
         <v>3420</v>
@@ -6027,10 +6027,10 @@
         <v>2370</v>
       </c>
       <c r="P29" s="148" t="n">
-        <v>1431</v>
+        <v>1428.090909090909</v>
       </c>
       <c r="Q29" s="140" t="n">
-        <v>0.548501742160279</v>
+        <v>0.5473519163763066</v>
       </c>
       <c r="R29" s="150" t="inlineStr">
         <is>
@@ -6086,25 +6086,25 @@
         <v>5</v>
       </c>
       <c r="K30" s="154" t="n">
-        <v>370</v>
+        <v>368.5</v>
       </c>
       <c r="L30" s="154" t="n">
-        <v>530</v>
+        <v>528.5</v>
       </c>
       <c r="M30" s="154" t="n">
-        <v>1210</v>
+        <v>1560</v>
       </c>
       <c r="N30" s="154" t="n">
-        <v>1000</v>
+        <v>1290</v>
       </c>
       <c r="O30" s="154" t="n">
-        <v>800</v>
+        <v>1030</v>
       </c>
       <c r="P30" s="139" t="n">
-        <v>379</v>
+        <v>644.2272727272725</v>
       </c>
       <c r="Q30" s="155" t="n">
-        <v>0.417</v>
+        <v>0.5493410852713178</v>
       </c>
       <c r="R30" s="153" t="inlineStr">
         <is>
@@ -6160,10 +6160,10 @@
         <v>5</v>
       </c>
       <c r="K31" s="154" t="n">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="L31" s="154" t="n">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="M31" s="154" t="n">
         <v>1710</v>
@@ -6175,10 +6175,10 @@
         <v>1100</v>
       </c>
       <c r="P31" s="147" t="n">
-        <v>635</v>
+        <v>635.5454545454545</v>
       </c>
       <c r="Q31" s="140" t="n">
-        <v>0.505797101449275</v>
+        <v>0.5065942028985507</v>
       </c>
       <c r="R31" s="153" t="inlineStr">
         <is>
@@ -6234,10 +6234,10 @@
         <v>5</v>
       </c>
       <c r="K32" s="154" t="n">
-        <v>590</v>
+        <v>586.5</v>
       </c>
       <c r="L32" s="154" t="n">
-        <v>815</v>
+        <v>811.5</v>
       </c>
       <c r="M32" s="154" t="n">
         <v>3090</v>
@@ -6249,10 +6249,10 @@
         <v>2040</v>
       </c>
       <c r="P32" s="148" t="n">
-        <v>1385</v>
+        <v>1388.5</v>
       </c>
       <c r="Q32" s="145" t="n">
-        <v>0.629545454545455</v>
+        <v>0.6311363636363636</v>
       </c>
       <c r="R32" s="153" t="inlineStr">
         <is>
@@ -6314,19 +6314,19 @@
         <v>218</v>
       </c>
       <c r="M33" s="154" t="n">
-        <v>550</v>
+        <v>760</v>
       </c>
       <c r="N33" s="154" t="n">
-        <v>490</v>
+        <v>680</v>
       </c>
       <c r="O33" s="154" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="P33" s="147" t="n">
-        <v>227</v>
+        <v>400.1818181818181</v>
       </c>
       <c r="Q33" s="140" t="n">
-        <v>0.510612244897959</v>
+        <v>0.6473529411764706</v>
       </c>
       <c r="R33" s="153" t="inlineStr">
         <is>
@@ -6382,25 +6382,25 @@
         <v>0</v>
       </c>
       <c r="K34" s="154" t="n">
-        <v>110</v>
+        <v>110.25</v>
       </c>
       <c r="L34" s="154" t="n">
-        <v>165</v>
+        <v>165.25</v>
       </c>
       <c r="M34" s="154" t="n">
-        <v>530</v>
+        <v>730</v>
       </c>
       <c r="N34" s="154" t="n">
-        <v>420</v>
+        <v>580</v>
       </c>
       <c r="O34" s="154" t="n">
-        <v>320</v>
+        <v>440</v>
       </c>
       <c r="P34" s="139" t="n">
-        <v>217</v>
+        <v>362.0227272727273</v>
       </c>
       <c r="Q34" s="145" t="n">
-        <v>0.5678571428571429</v>
+        <v>0.6865948275862069</v>
       </c>
       <c r="R34" s="153" t="inlineStr">
         <is>
@@ -6456,10 +6456,10 @@
         <v>0</v>
       </c>
       <c r="K35" s="154" t="n">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L35" s="154" t="n">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="M35" s="154" t="n">
         <v>890</v>
@@ -6471,10 +6471,10 @@
         <v>580</v>
       </c>
       <c r="P35" s="147" t="n">
-        <v>410</v>
+        <v>410.5454545454545</v>
       </c>
       <c r="Q35" s="145" t="n">
-        <v>0.625694444444444</v>
+        <v>0.6272222222222222</v>
       </c>
       <c r="R35" s="153" t="inlineStr">
         <is>
@@ -6530,25 +6530,25 @@
         <v>5</v>
       </c>
       <c r="K36" s="154" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L36" s="154" t="n">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="M36" s="154" t="n">
-        <v>830</v>
+        <v>1060</v>
       </c>
       <c r="N36" s="154" t="n">
-        <v>660</v>
+        <v>840</v>
       </c>
       <c r="O36" s="154" t="n">
-        <v>530</v>
+        <v>670</v>
       </c>
       <c r="P36" s="139" t="n">
-        <v>300</v>
+        <v>462.6363636363636</v>
       </c>
       <c r="Q36" s="140" t="n">
-        <v>0.5</v>
+        <v>0.6058333333333333</v>
       </c>
       <c r="R36" s="153" t="inlineStr">
         <is>
@@ -6619,10 +6619,10 @@
         <v>690</v>
       </c>
       <c r="P37" s="147" t="n">
-        <v>422</v>
+        <v>421.8181818181818</v>
       </c>
       <c r="Q37" s="140" t="n">
-        <v>0.5395348837209299</v>
+        <v>0.5395348837209302</v>
       </c>
       <c r="R37" s="153" t="inlineStr">
         <is>
@@ -6684,19 +6684,19 @@
         <v>85</v>
       </c>
       <c r="M38" s="158" t="n">
-        <v>280</v>
+        <v>510</v>
       </c>
       <c r="N38" s="158" t="n">
-        <v>230</v>
+        <v>420</v>
       </c>
       <c r="O38" s="158" t="n">
-        <v>170</v>
+        <v>310</v>
       </c>
       <c r="P38" s="139" t="n">
-        <v>124</v>
+        <v>296.8181818181818</v>
       </c>
       <c r="Q38" s="145" t="n">
-        <v>0.593478260869565</v>
+        <v>0.7773809523809524</v>
       </c>
       <c r="R38" s="157" t="inlineStr">
         <is>
@@ -6758,19 +6758,19 @@
         <v>65</v>
       </c>
       <c r="M39" s="158" t="n">
-        <v>230</v>
+        <v>490</v>
       </c>
       <c r="N39" s="158" t="n">
-        <v>180</v>
+        <v>380</v>
       </c>
       <c r="O39" s="158" t="n">
-        <v>140</v>
+        <v>300</v>
       </c>
       <c r="P39" s="139" t="n">
-        <v>99</v>
+        <v>280.4545454545454</v>
       </c>
       <c r="Q39" s="145" t="n">
-        <v>0.602777777777778</v>
+        <v>0.8118421052631579</v>
       </c>
       <c r="R39" s="157" t="inlineStr">
         <is>
@@ -6915,10 +6915,10 @@
         <v>2370</v>
       </c>
       <c r="P41" s="148" t="n">
-        <v>1436</v>
+        <v>1436.090909090909</v>
       </c>
       <c r="Q41" s="145" t="n">
-        <v>0.550418118466899</v>
+        <v>0.5504181184668989</v>
       </c>
       <c r="R41" s="160" t="inlineStr">
         <is>
@@ -6974,10 +6974,10 @@
         <v>63</v>
       </c>
       <c r="K42" s="161" t="n">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="L42" s="161" t="n">
-        <v>1393</v>
+        <v>1391</v>
       </c>
       <c r="M42" s="161" t="n">
         <v>3970</v>
@@ -6989,10 +6989,10 @@
         <v>2700</v>
       </c>
       <c r="P42" s="162" t="n">
-        <v>1516</v>
+        <v>1518.090909090909</v>
       </c>
       <c r="Q42" s="140" t="n">
-        <v>0.52115625</v>
+        <v>0.5218437499999999</v>
       </c>
       <c r="R42" s="160" t="inlineStr">
         <is>
@@ -7048,10 +7048,10 @@
         <v>63</v>
       </c>
       <c r="K43" s="161" t="n">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="L43" s="161" t="n">
-        <v>1493</v>
+        <v>1497</v>
       </c>
       <c r="M43" s="161" t="n">
         <v>4290</v>
@@ -7063,10 +7063,10 @@
         <v>2980</v>
       </c>
       <c r="P43" s="162" t="n">
-        <v>1716</v>
+        <v>1712.090909090909</v>
       </c>
       <c r="Q43" s="140" t="n">
-        <v>0.534759206798867</v>
+        <v>0.5335127478753541</v>
       </c>
       <c r="R43" s="160" t="inlineStr">
         <is>
@@ -7122,10 +7122,10 @@
         <v>53</v>
       </c>
       <c r="K44" s="161" t="n">
-        <v>840</v>
+        <v>836</v>
       </c>
       <c r="L44" s="161" t="n">
-        <v>1288</v>
+        <v>1284</v>
       </c>
       <c r="M44" s="161" t="n">
         <v>3750</v>
@@ -7137,10 +7137,10 @@
         <v>2590</v>
       </c>
       <c r="P44" s="162" t="n">
-        <v>1521</v>
+        <v>1525.090909090909</v>
       </c>
       <c r="Q44" s="140" t="n">
-        <v>0.541488673139159</v>
+        <v>0.5429126213592232</v>
       </c>
       <c r="R44" s="160" t="inlineStr">
         <is>
@@ -7196,10 +7196,10 @@
         <v>73</v>
       </c>
       <c r="K45" s="161" t="n">
-        <v>1300</v>
+        <v>1305</v>
       </c>
       <c r="L45" s="161" t="n">
-        <v>1903</v>
+        <v>1908</v>
       </c>
       <c r="M45" s="161" t="n">
         <v>5730</v>
@@ -7211,10 +7211,10 @@
         <v>3970</v>
       </c>
       <c r="P45" s="162" t="n">
-        <v>2297</v>
+        <v>2292</v>
       </c>
       <c r="Q45" s="140" t="n">
-        <v>0.546904761904762</v>
+        <v>0.5457142857142857</v>
       </c>
       <c r="R45" s="160" t="inlineStr">
         <is>
@@ -7270,10 +7270,10 @@
         <v>48</v>
       </c>
       <c r="K46" s="161" t="n">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="L46" s="161" t="n">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="M46" s="161" t="n">
         <v>2310</v>
@@ -7285,10 +7285,10 @@
         <v>1550</v>
       </c>
       <c r="P46" s="148" t="n">
-        <v>972</v>
+        <v>970.5454545454545</v>
       </c>
       <c r="Q46" s="145" t="n">
-        <v>0.553730569948187</v>
+        <v>0.553160621761658</v>
       </c>
       <c r="R46" s="160" t="inlineStr">
         <is>
@@ -7359,10 +7359,10 @@
         <v>1880</v>
       </c>
       <c r="P47" s="148" t="n">
-        <v>1150</v>
+        <v>1149.545454545455</v>
       </c>
       <c r="Q47" s="145" t="n">
-        <v>0.559513274336283</v>
+        <v>0.5595132743362832</v>
       </c>
       <c r="R47" s="160" t="inlineStr">
         <is>
@@ -7418,10 +7418,10 @@
         <v>5</v>
       </c>
       <c r="K48" s="161" t="n">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="L48" s="161" t="n">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="M48" s="161" t="n">
         <v>1660</v>
@@ -7433,10 +7433,10 @@
         <v>1080</v>
       </c>
       <c r="P48" s="147" t="n">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="Q48" s="155" t="n">
-        <v>0.415833333333333</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="R48" s="160" t="inlineStr">
         <is>
@@ -7492,10 +7492,10 @@
         <v>5</v>
       </c>
       <c r="K49" s="161" t="n">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="L49" s="161" t="n">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="M49" s="161" t="n">
         <v>2090</v>
@@ -7507,10 +7507,10 @@
         <v>1380</v>
       </c>
       <c r="P49" s="147" t="n">
-        <v>732</v>
+        <v>733.5454545454545</v>
       </c>
       <c r="Q49" s="140" t="n">
-        <v>0.470584795321637</v>
+        <v>0.4718713450292398</v>
       </c>
       <c r="R49" s="160" t="inlineStr">
         <is>
@@ -7640,10 +7640,10 @@
         <v>53</v>
       </c>
       <c r="K51" s="165" t="n">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="L51" s="165" t="n">
-        <v>1328</v>
+        <v>1332</v>
       </c>
       <c r="M51" s="165" t="n">
         <v>3970</v>
@@ -7655,10 +7655,10 @@
         <v>2640</v>
       </c>
       <c r="P51" s="162" t="n">
-        <v>1581</v>
+        <v>1577.090909090909</v>
       </c>
       <c r="Q51" s="140" t="n">
-        <v>0.5435</v>
+        <v>0.542125</v>
       </c>
       <c r="R51" s="164" t="inlineStr">
         <is>
@@ -7714,10 +7714,10 @@
         <v>53</v>
       </c>
       <c r="K52" s="165" t="n">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="L52" s="165" t="n">
-        <v>1413</v>
+        <v>1409</v>
       </c>
       <c r="M52" s="165" t="n">
         <v>4290</v>
@@ -7729,10 +7729,10 @@
         <v>2920</v>
       </c>
       <c r="P52" s="162" t="n">
-        <v>1796</v>
+        <v>1800.090909090909</v>
       </c>
       <c r="Q52" s="145" t="n">
-        <v>0.559688385269122</v>
+        <v>0.5609348441926345</v>
       </c>
       <c r="R52" s="164" t="inlineStr">
         <is>
@@ -7803,10 +7803,10 @@
         <v>3310</v>
       </c>
       <c r="P53" s="162" t="n">
-        <v>1901</v>
+        <v>1901.090909090909</v>
       </c>
       <c r="Q53" s="140" t="n">
-        <v>0.526750629722922</v>
+        <v>0.5267506297229219</v>
       </c>
       <c r="R53" s="164" t="inlineStr">
         <is>
@@ -7862,10 +7862,10 @@
         <v>58</v>
       </c>
       <c r="K54" s="165" t="n">
-        <v>1220</v>
+        <v>1216</v>
       </c>
       <c r="L54" s="165" t="n">
-        <v>1798</v>
+        <v>1794</v>
       </c>
       <c r="M54" s="165" t="n">
         <v>5280</v>
@@ -7877,10 +7877,10 @@
         <v>3640</v>
       </c>
       <c r="P54" s="162" t="n">
-        <v>2102</v>
+        <v>2106</v>
       </c>
       <c r="Q54" s="140" t="n">
-        <v>0.538974358974359</v>
+        <v>0.5399999999999999</v>
       </c>
       <c r="R54" s="164" t="inlineStr">
         <is>
@@ -7936,10 +7936,10 @@
         <v>73</v>
       </c>
       <c r="K55" s="165" t="n">
-        <v>1500</v>
+        <v>1494</v>
       </c>
       <c r="L55" s="165" t="n">
-        <v>2083</v>
+        <v>2077</v>
       </c>
       <c r="M55" s="165" t="n">
         <v>7160</v>
@@ -7951,10 +7951,10 @@
         <v>4840</v>
       </c>
       <c r="P55" s="162" t="n">
-        <v>3126</v>
+        <v>3132.090909090909</v>
       </c>
       <c r="Q55" s="145" t="n">
-        <v>0.600122164048866</v>
+        <v>0.6012739965095986</v>
       </c>
       <c r="R55" s="164" t="inlineStr">
         <is>
@@ -8010,10 +8010,10 @@
         <v>73</v>
       </c>
       <c r="K56" s="165" t="n">
-        <v>1580</v>
+        <v>1577</v>
       </c>
       <c r="L56" s="165" t="n">
-        <v>2173</v>
+        <v>2170</v>
       </c>
       <c r="M56" s="165" t="n">
         <v>7710</v>
@@ -8025,10 +8025,10 @@
         <v>5280</v>
       </c>
       <c r="P56" s="162" t="n">
-        <v>3436</v>
+        <v>3439.090909090909</v>
       </c>
       <c r="Q56" s="145" t="n">
-        <v>0.61259319286872</v>
+        <v>0.613128038897893</v>
       </c>
       <c r="R56" s="164" t="inlineStr">
         <is>
@@ -8084,10 +8084,10 @@
         <v>50</v>
       </c>
       <c r="K57" s="161" t="n">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="L57" s="161" t="n">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="M57" s="161" t="n">
         <v>2870</v>
@@ -8099,10 +8099,10 @@
         <v>1930</v>
       </c>
       <c r="P57" s="148" t="n">
-        <v>1185</v>
+        <v>1188.545454545455</v>
       </c>
       <c r="Q57" s="140" t="n">
-        <v>0.5497890295358649</v>
+        <v>0.5516455696202531</v>
       </c>
       <c r="R57" s="160" t="inlineStr">
         <is>
@@ -8158,10 +8158,10 @@
         <v>8</v>
       </c>
       <c r="K58" s="161" t="n">
-        <v>450</v>
+        <v>448.5</v>
       </c>
       <c r="L58" s="161" t="n">
-        <v>656</v>
+        <v>654.5</v>
       </c>
       <c r="M58" s="161" t="n">
         <v>1880</v>
@@ -8173,10 +8173,10 @@
         <v>1210</v>
       </c>
       <c r="P58" s="147" t="n">
-        <v>753</v>
+        <v>754.590909090909</v>
       </c>
       <c r="Q58" s="140" t="n">
-        <v>0.534451612903226</v>
+        <v>0.5355161290322581</v>
       </c>
       <c r="R58" s="160" t="inlineStr">
         <is>
@@ -8247,10 +8247,10 @@
         <v>1600</v>
       </c>
       <c r="P59" s="148" t="n">
-        <v>1020</v>
+        <v>1020.090909090909</v>
       </c>
       <c r="Q59" s="145" t="n">
-        <v>0.563869346733668</v>
+        <v>0.5638693467336683</v>
       </c>
       <c r="R59" s="160" t="inlineStr">
         <is>
@@ -8324,7 +8324,7 @@
         <v>607</v>
       </c>
       <c r="Q60" s="145" t="n">
-        <v>0.551818181818182</v>
+        <v>0.5518181818181818</v>
       </c>
       <c r="R60" s="167" t="inlineStr">
         <is>
@@ -8380,10 +8380,10 @@
         <v>46</v>
       </c>
       <c r="K61" s="168" t="n">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="L61" s="168" t="n">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="M61" s="168" t="n">
         <v>1880</v>
@@ -8395,10 +8395,10 @@
         <v>1210</v>
       </c>
       <c r="P61" s="147" t="n">
-        <v>740</v>
+        <v>738.090909090909</v>
       </c>
       <c r="Q61" s="140" t="n">
-        <v>0.525225806451613</v>
+        <v>0.5238064516129032</v>
       </c>
       <c r="R61" s="167" t="inlineStr">
         <is>
@@ -8602,10 +8602,10 @@
         <v>30</v>
       </c>
       <c r="K64" s="144" t="n">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="L64" s="144" t="n">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="M64" s="144" t="n">
         <v>1000</v>
@@ -8617,10 +8617,10 @@
         <v>660</v>
       </c>
       <c r="P64" s="147" t="n">
-        <v>423</v>
+        <v>423.5454545454545</v>
       </c>
       <c r="Q64" s="145" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5613253012048193</v>
       </c>
       <c r="R64" s="143" t="inlineStr">
         <is>
@@ -8676,10 +8676,10 @@
         <v>35</v>
       </c>
       <c r="K65" s="144" t="n">
-        <v>300</v>
+        <v>301.5</v>
       </c>
       <c r="L65" s="144" t="n">
-        <v>400</v>
+        <v>401.5</v>
       </c>
       <c r="M65" s="144" t="n">
         <v>1440</v>
@@ -8691,10 +8691,10 @@
         <v>940</v>
       </c>
       <c r="P65" s="147" t="n">
-        <v>655</v>
+        <v>653.0454545454545</v>
       </c>
       <c r="Q65" s="145" t="n">
-        <v>0.620689655172414</v>
+        <v>0.6192672413793103</v>
       </c>
       <c r="R65" s="143" t="inlineStr">
         <is>
@@ -8750,10 +8750,10 @@
         <v>35</v>
       </c>
       <c r="K66" s="144" t="n">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="L66" s="144" t="n">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="M66" s="144" t="n">
         <v>1710</v>
@@ -8765,10 +8765,10 @@
         <v>1100</v>
       </c>
       <c r="P66" s="147" t="n">
-        <v>730</v>
+        <v>727.5454545454545</v>
       </c>
       <c r="Q66" s="145" t="n">
-        <v>0.581521739130435</v>
+        <v>0.5799275362318841</v>
       </c>
       <c r="R66" s="143" t="inlineStr">
         <is>
@@ -8843,7 +8843,7 @@
         <v>555</v>
       </c>
       <c r="Q67" s="140" t="n">
-        <v>0.504545454545455</v>
+        <v>0.5045454545454545</v>
       </c>
       <c r="R67" s="170" t="inlineStr">
         <is>
@@ -8900,10 +8900,10 @@
         <v>5</v>
       </c>
       <c r="K68" s="172" t="n">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="L68" s="172" t="n">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="M68" s="172" t="n">
         <v>1770</v>
@@ -8915,10 +8915,10 @@
         <v>1210</v>
       </c>
       <c r="P68" s="173" t="n">
-        <v>760</v>
+        <v>757.5454545454545</v>
       </c>
       <c r="Q68" s="174" t="n">
-        <v>0.560738255033557</v>
+        <v>0.559261744966443</v>
       </c>
       <c r="R68" s="170" t="inlineStr">
         <is>
@@ -8990,7 +8990,7 @@
         <v>1490</v>
       </c>
       <c r="P69" s="148" t="n">
-        <v>980</v>
+        <v>979.5454545454545</v>
       </c>
       <c r="Q69" s="145" t="n">
         <v>0.592032967032967</v>
@@ -9049,10 +9049,10 @@
         <v>5</v>
       </c>
       <c r="K70" s="171" t="n">
-        <v>420</v>
+        <v>422.5</v>
       </c>
       <c r="L70" s="171" t="n">
-        <v>705</v>
+        <v>707.5</v>
       </c>
       <c r="M70" s="171" t="n">
         <v>1880</v>
@@ -9064,10 +9064,10 @@
         <v>1210</v>
       </c>
       <c r="P70" s="147" t="n">
-        <v>704</v>
+        <v>701.590909090909</v>
       </c>
       <c r="Q70" s="140" t="n">
-        <v>0.499677419354839</v>
+        <v>0.4979032258064516</v>
       </c>
       <c r="R70" s="170" t="inlineStr">
         <is>
@@ -9138,10 +9138,10 @@
         <v>1490</v>
       </c>
       <c r="P71" s="148" t="n">
-        <v>890</v>
+        <v>889.5454545454545</v>
       </c>
       <c r="Q71" s="140" t="n">
-        <v>0.5376373626373629</v>
+        <v>0.5376373626373626</v>
       </c>
       <c r="R71" s="170" t="inlineStr">
         <is>
@@ -9197,10 +9197,10 @@
         <v>5</v>
       </c>
       <c r="K72" s="171" t="n">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="L72" s="171" t="n">
-        <v>865</v>
+        <v>861</v>
       </c>
       <c r="M72" s="171" t="n">
         <v>2640</v>
@@ -9212,10 +9212,10 @@
         <v>1770</v>
       </c>
       <c r="P72" s="148" t="n">
-        <v>1090</v>
+        <v>1093.545454545454</v>
       </c>
       <c r="Q72" s="145" t="n">
-        <v>0.557441860465116</v>
+        <v>0.5594883720930232</v>
       </c>
       <c r="R72" s="170" t="inlineStr">
         <is>
@@ -9286,7 +9286,7 @@
         <v>780</v>
       </c>
       <c r="P73" s="147" t="n">
-        <v>464</v>
+        <v>464.090909090909</v>
       </c>
       <c r="Q73" s="140" t="n">
         <v>0.5105</v>
@@ -9363,7 +9363,7 @@
         <v>595</v>
       </c>
       <c r="Q74" s="140" t="n">
-        <v>0.540909090909091</v>
+        <v>0.5409090909090909</v>
       </c>
       <c r="R74" s="170" t="inlineStr">
         <is>
@@ -9419,10 +9419,10 @@
         <v>5</v>
       </c>
       <c r="K75" s="171" t="n">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="L75" s="171" t="n">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="M75" s="171" t="n">
         <v>1880</v>
@@ -9434,10 +9434,10 @@
         <v>1210</v>
       </c>
       <c r="P75" s="148" t="n">
-        <v>814</v>
+        <v>815.090909090909</v>
       </c>
       <c r="Q75" s="145" t="n">
-        <v>0.577741935483871</v>
+        <v>0.5784516129032258</v>
       </c>
       <c r="R75" s="170" t="inlineStr">
         <is>
@@ -9494,10 +9494,10 @@
         <v>5</v>
       </c>
       <c r="K76" s="171" t="n">
-        <v>380</v>
+        <v>379.5</v>
       </c>
       <c r="L76" s="171" t="n">
-        <v>585</v>
+        <v>584.5</v>
       </c>
       <c r="M76" s="171" t="n">
         <v>1660</v>
@@ -9509,10 +9509,10 @@
         <v>1050</v>
       </c>
       <c r="P76" s="147" t="n">
-        <v>615</v>
+        <v>615.5</v>
       </c>
       <c r="Q76" s="140" t="n">
-        <v>0.5125</v>
+        <v>0.5129166666666667</v>
       </c>
       <c r="R76" s="170" t="inlineStr">
         <is>
@@ -9569,10 +9569,10 @@
         <v>5</v>
       </c>
       <c r="K77" s="171" t="n">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="L77" s="171" t="n">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="M77" s="171" t="n">
         <v>2420</v>
@@ -9584,10 +9584,10 @@
         <v>1600</v>
       </c>
       <c r="P77" s="148" t="n">
-        <v>1054</v>
+        <v>1052.090909090909</v>
       </c>
       <c r="Q77" s="145" t="n">
-        <v>0.582663316582915</v>
+        <v>0.5815577889447237</v>
       </c>
       <c r="R77" s="170" t="inlineStr">
         <is>
@@ -9719,10 +9719,10 @@
         <v>8</v>
       </c>
       <c r="K79" s="171" t="n">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="L79" s="171" t="n">
-        <v>1208</v>
+        <v>1203</v>
       </c>
       <c r="M79" s="171" t="n">
         <v>3860</v>
@@ -9734,10 +9734,10 @@
         <v>2530</v>
       </c>
       <c r="P79" s="162" t="n">
-        <v>1601</v>
+        <v>1606.090909090909</v>
       </c>
       <c r="Q79" s="145" t="n">
-        <v>0.569967637540453</v>
+        <v>0.571747572815534</v>
       </c>
       <c r="R79" s="170" t="inlineStr">
         <is>
@@ -9794,10 +9794,10 @@
         <v>10</v>
       </c>
       <c r="K80" s="171" t="n">
-        <v>1100</v>
+        <v>1104</v>
       </c>
       <c r="L80" s="171" t="n">
-        <v>1460</v>
+        <v>1464</v>
       </c>
       <c r="M80" s="171" t="n">
         <v>4950</v>
@@ -9809,10 +9809,10 @@
         <v>3310</v>
       </c>
       <c r="P80" s="162" t="n">
-        <v>2149</v>
+        <v>2145.090909090909</v>
       </c>
       <c r="Q80" s="145" t="n">
-        <v>0.595465994962217</v>
+        <v>0.5943576826196474</v>
       </c>
       <c r="R80" s="170" t="inlineStr">
         <is>
@@ -9886,7 +9886,7 @@
         <v>1252</v>
       </c>
       <c r="Q81" s="140" t="n">
-        <v>0.544347826086957</v>
+        <v>0.5443478260869565</v>
       </c>
       <c r="R81" s="176" t="inlineStr">
         <is>
@@ -9942,10 +9942,10 @@
         <v>8</v>
       </c>
       <c r="K82" s="177" t="n">
-        <v>920</v>
+        <v>923</v>
       </c>
       <c r="L82" s="177" t="n">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="M82" s="177" t="n">
         <v>3860</v>
@@ -9957,10 +9957,10 @@
         <v>2640</v>
       </c>
       <c r="P82" s="162" t="n">
-        <v>1661</v>
+        <v>1658.090909090909</v>
       </c>
       <c r="Q82" s="145" t="n">
-        <v>0.571</v>
+        <v>0.56996875</v>
       </c>
       <c r="R82" s="176" t="inlineStr">
         <is>
@@ -10031,7 +10031,7 @@
         <v>3090</v>
       </c>
       <c r="P83" s="162" t="n">
-        <v>2029</v>
+        <v>2029.090909090909</v>
       </c>
       <c r="Q83" s="145" t="n">
         <v>0.5952</v>
@@ -10090,10 +10090,10 @@
         <v>10</v>
       </c>
       <c r="K84" s="177" t="n">
-        <v>1400</v>
+        <v>1404</v>
       </c>
       <c r="L84" s="177" t="n">
-        <v>1730</v>
+        <v>1734</v>
       </c>
       <c r="M84" s="177" t="n">
         <v>6060</v>
@@ -10105,10 +10105,10 @@
         <v>4180</v>
       </c>
       <c r="P84" s="162" t="n">
-        <v>2770</v>
+        <v>2766</v>
       </c>
       <c r="Q84" s="145" t="n">
-        <v>0.615555555555556</v>
+        <v>0.6146666666666667</v>
       </c>
       <c r="R84" s="176" t="inlineStr">
         <is>
@@ -10164,10 +10164,10 @@
         <v>53</v>
       </c>
       <c r="K85" s="177" t="n">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="L85" s="177" t="n">
-        <v>1113</v>
+        <v>1117</v>
       </c>
       <c r="M85" s="177" t="n">
         <v>3530</v>
@@ -10179,10 +10179,10 @@
         <v>2370</v>
       </c>
       <c r="P85" s="148" t="n">
-        <v>1496</v>
+        <v>1492.090909090909</v>
       </c>
       <c r="Q85" s="145" t="n">
-        <v>0.573414634146341</v>
+        <v>0.5718815331010453</v>
       </c>
       <c r="R85" s="176" t="inlineStr">
         <is>
@@ -10238,10 +10238,10 @@
         <v>53</v>
       </c>
       <c r="K86" s="177" t="n">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="L86" s="177" t="n">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="M86" s="177" t="n">
         <v>3200</v>
@@ -10253,10 +10253,10 @@
         <v>2150</v>
       </c>
       <c r="P86" s="148" t="n">
-        <v>1347</v>
+        <v>1350</v>
       </c>
       <c r="Q86" s="145" t="n">
-        <v>0.56125</v>
+        <v>0.5625</v>
       </c>
       <c r="R86" s="176" t="inlineStr">
         <is>
@@ -10312,10 +10312,10 @@
         <v>63</v>
       </c>
       <c r="K87" s="177" t="n">
-        <v>1500</v>
+        <v>1494</v>
       </c>
       <c r="L87" s="177" t="n">
-        <v>1823</v>
+        <v>1817</v>
       </c>
       <c r="M87" s="177" t="n">
         <v>6610</v>
@@ -10327,10 +10327,10 @@
         <v>4400</v>
       </c>
       <c r="P87" s="162" t="n">
-        <v>2977</v>
+        <v>2983</v>
       </c>
       <c r="Q87" s="145" t="n">
-        <v>0.620208333333333</v>
+        <v>0.6214583333333333</v>
       </c>
       <c r="R87" s="176" t="inlineStr">
         <is>
@@ -10392,19 +10392,19 @@
         <v>105</v>
       </c>
       <c r="M88" s="158" t="n">
-        <v>360</v>
+        <v>490</v>
       </c>
       <c r="N88" s="158" t="n">
-        <v>280</v>
+        <v>380</v>
       </c>
       <c r="O88" s="158" t="n">
-        <v>230</v>
+        <v>310</v>
       </c>
       <c r="P88" s="139" t="n">
-        <v>150</v>
+        <v>240.4545454545454</v>
       </c>
       <c r="Q88" s="145" t="n">
-        <v>0.5875</v>
+        <v>0.6960526315789474</v>
       </c>
       <c r="R88" s="157" t="inlineStr">
         <is>
@@ -10460,25 +10460,25 @@
         <v>0</v>
       </c>
       <c r="K89" s="158" t="n">
-        <v>110</v>
+        <v>109.5</v>
       </c>
       <c r="L89" s="158" t="n">
-        <v>145</v>
+        <v>144.5</v>
       </c>
       <c r="M89" s="158" t="n">
-        <v>470</v>
+        <v>650</v>
       </c>
       <c r="N89" s="158" t="n">
-        <v>390</v>
+        <v>540</v>
       </c>
       <c r="O89" s="158" t="n">
-        <v>310</v>
+        <v>430</v>
       </c>
       <c r="P89" s="139" t="n">
-        <v>210</v>
+        <v>346.4090909090909</v>
       </c>
       <c r="Q89" s="145" t="n">
-        <v>0.591025641025641</v>
+        <v>0.7056481481481481</v>
       </c>
       <c r="R89" s="157" t="inlineStr">
         <is>
@@ -10540,19 +10540,19 @@
         <v>80</v>
       </c>
       <c r="M90" s="158" t="n">
-        <v>280</v>
+        <v>500</v>
       </c>
       <c r="N90" s="158" t="n">
-        <v>230</v>
+        <v>410</v>
       </c>
       <c r="O90" s="158" t="n">
-        <v>170</v>
+        <v>300</v>
       </c>
       <c r="P90" s="139" t="n">
-        <v>129</v>
+        <v>292.7272727272727</v>
       </c>
       <c r="Q90" s="145" t="n">
-        <v>0.617391304347826</v>
+        <v>0.7853658536585366</v>
       </c>
       <c r="R90" s="157" t="inlineStr">
         <is>
@@ -10614,19 +10614,19 @@
         <v>78</v>
       </c>
       <c r="M91" s="178" t="n">
-        <v>280</v>
+        <v>500</v>
       </c>
       <c r="N91" s="178" t="n">
-        <v>230</v>
+        <v>410</v>
       </c>
       <c r="O91" s="178" t="n">
-        <v>170</v>
+        <v>300</v>
       </c>
       <c r="P91" s="179" t="n">
-        <v>131</v>
+        <v>294.7272727272727</v>
       </c>
       <c r="Q91" s="174" t="n">
-        <v>0.62695652173913</v>
+        <v>0.7907317073170731</v>
       </c>
       <c r="R91" s="157" t="inlineStr">
         <is>
@@ -10682,25 +10682,25 @@
         <v>0</v>
       </c>
       <c r="K92" s="158" t="n">
-        <v>100</v>
+        <v>100.5</v>
       </c>
       <c r="L92" s="158" t="n">
-        <v>130</v>
+        <v>130.5</v>
       </c>
       <c r="M92" s="158" t="n">
+        <v>650</v>
+      </c>
+      <c r="N92" s="158" t="n">
+        <v>510</v>
+      </c>
+      <c r="O92" s="158" t="n">
         <v>420</v>
       </c>
-      <c r="N92" s="158" t="n">
-        <v>330</v>
-      </c>
-      <c r="O92" s="158" t="n">
-        <v>270</v>
-      </c>
       <c r="P92" s="139" t="n">
-        <v>170</v>
+        <v>333.1363636363636</v>
       </c>
       <c r="Q92" s="145" t="n">
-        <v>0.566666666666667</v>
+        <v>0.7185294117647059</v>
       </c>
       <c r="R92" s="157" t="inlineStr">
         <is>
@@ -10762,19 +10762,19 @@
         <v>510</v>
       </c>
       <c r="M93" s="154" t="n">
-        <v>1160</v>
+        <v>1540</v>
       </c>
       <c r="N93" s="154" t="n">
-        <v>940</v>
+        <v>1250</v>
       </c>
       <c r="O93" s="154" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="P93" s="139" t="n">
-        <v>345</v>
+        <v>626.3636363636363</v>
       </c>
       <c r="Q93" s="155" t="n">
-        <v>0.403191489361702</v>
+        <v>0.5511999999999999</v>
       </c>
       <c r="R93" s="153" t="inlineStr">
         <is>
@@ -10830,25 +10830,25 @@
         <v>5</v>
       </c>
       <c r="K94" s="154" t="n">
-        <v>370</v>
+        <v>368.5</v>
       </c>
       <c r="L94" s="154" t="n">
-        <v>530</v>
+        <v>528.5</v>
       </c>
       <c r="M94" s="154" t="n">
-        <v>1210</v>
+        <v>1560</v>
       </c>
       <c r="N94" s="154" t="n">
-        <v>1000</v>
+        <v>1290</v>
       </c>
       <c r="O94" s="154" t="n">
-        <v>800</v>
+        <v>1030</v>
       </c>
       <c r="P94" s="139" t="n">
-        <v>379</v>
+        <v>644.2272727272725</v>
       </c>
       <c r="Q94" s="155" t="n">
-        <v>0.417</v>
+        <v>0.5493410852713178</v>
       </c>
       <c r="R94" s="153" t="inlineStr">
         <is>
@@ -10904,10 +10904,10 @@
         <v>5</v>
       </c>
       <c r="K95" s="154" t="n">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="L95" s="154" t="n">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="M95" s="154" t="n">
         <v>1490</v>
@@ -10919,10 +10919,10 @@
         <v>970</v>
       </c>
       <c r="P95" s="147" t="n">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="Q95" s="155" t="n">
-        <v>0.404545454545455</v>
+        <v>0.4063636363636364</v>
       </c>
       <c r="R95" s="153" t="inlineStr">
         <is>
@@ -10978,25 +10978,25 @@
         <v>5</v>
       </c>
       <c r="K96" s="154" t="n">
-        <v>320</v>
+        <v>319.5</v>
       </c>
       <c r="L96" s="154" t="n">
-        <v>480</v>
+        <v>479.5</v>
       </c>
       <c r="M96" s="154" t="n">
-        <v>1050</v>
+        <v>1450</v>
       </c>
       <c r="N96" s="154" t="n">
-        <v>860</v>
+        <v>1190</v>
       </c>
       <c r="O96" s="154" t="n">
-        <v>690</v>
+        <v>950</v>
       </c>
       <c r="P96" s="139" t="n">
-        <v>302</v>
+        <v>602.3181818181818</v>
       </c>
       <c r="Q96" s="155" t="n">
-        <v>0.386046511627907</v>
+        <v>0.5567647058823529</v>
       </c>
       <c r="R96" s="153" t="inlineStr">
         <is>
@@ -11052,10 +11052,10 @@
         <v>5</v>
       </c>
       <c r="K97" s="154" t="n">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="L97" s="154" t="n">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="M97" s="154" t="n">
         <v>1770</v>
@@ -11067,10 +11067,10 @@
         <v>1160</v>
       </c>
       <c r="P97" s="147" t="n">
-        <v>624</v>
+        <v>621.090909090909</v>
       </c>
       <c r="Q97" s="140" t="n">
-        <v>0.476736111111111</v>
+        <v>0.4744444444444444</v>
       </c>
       <c r="R97" s="153" t="inlineStr">
         <is>
@@ -11126,10 +11126,10 @@
         <v>5</v>
       </c>
       <c r="K98" s="154" t="n">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="L98" s="154" t="n">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="M98" s="154" t="n">
         <v>2200</v>
@@ -11141,10 +11141,10 @@
         <v>1490</v>
       </c>
       <c r="P98" s="148" t="n">
-        <v>820</v>
+        <v>821.5454545454545</v>
       </c>
       <c r="Q98" s="140" t="n">
-        <v>0.49532967032967</v>
+        <v>0.4965384615384615</v>
       </c>
       <c r="R98" s="153" t="inlineStr">
         <is>
@@ -11200,10 +11200,10 @@
         <v>3</v>
       </c>
       <c r="K99" s="154" t="n">
-        <v>220</v>
+        <v>220.5</v>
       </c>
       <c r="L99" s="154" t="n">
-        <v>298</v>
+        <v>298.5</v>
       </c>
       <c r="M99" s="154" t="n">
         <v>940</v>
@@ -11215,10 +11215,10 @@
         <v>610</v>
       </c>
       <c r="P99" s="139" t="n">
-        <v>384</v>
+        <v>383.3181818181818</v>
       </c>
       <c r="Q99" s="145" t="n">
-        <v>0.562933333333333</v>
+        <v>0.5621999999999999</v>
       </c>
       <c r="R99" s="153" t="inlineStr">
         <is>
@@ -11280,19 +11280,19 @@
         <v>248</v>
       </c>
       <c r="M100" s="154" t="n">
-        <v>720</v>
+        <v>920</v>
       </c>
       <c r="N100" s="154" t="n">
-        <v>580</v>
+        <v>740</v>
       </c>
       <c r="O100" s="154" t="n">
-        <v>470</v>
+        <v>600</v>
       </c>
       <c r="P100" s="139" t="n">
-        <v>279</v>
+        <v>424.7272727272726</v>
       </c>
       <c r="Q100" s="140" t="n">
-        <v>0.529655172413793</v>
+        <v>0.6313513513513513</v>
       </c>
       <c r="R100" s="153" t="inlineStr">
         <is>
@@ -11366,7 +11366,7 @@
         <v>362</v>
       </c>
       <c r="Q101" s="145" t="n">
-        <v>0.6033333333333331</v>
+        <v>0.6033333333333334</v>
       </c>
       <c r="R101" s="157" t="inlineStr">
         <is>
@@ -11422,10 +11422,10 @@
         <v>3</v>
       </c>
       <c r="K102" s="158" t="n">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L102" s="158" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="M102" s="158" t="n">
         <v>1210</v>
@@ -11437,10 +11437,10 @@
         <v>800</v>
       </c>
       <c r="P102" s="147" t="n">
-        <v>541</v>
+        <v>542.090909090909</v>
       </c>
       <c r="Q102" s="145" t="n">
-        <v>0.5952</v>
+        <v>0.5962999999999999</v>
       </c>
       <c r="R102" s="157" t="inlineStr">
         <is>
@@ -11502,19 +11502,19 @@
         <v>150</v>
       </c>
       <c r="M103" s="158" t="n">
-        <v>500</v>
+        <v>710</v>
       </c>
       <c r="N103" s="158" t="n">
-        <v>390</v>
+        <v>550</v>
       </c>
       <c r="O103" s="158" t="n">
-        <v>310</v>
+        <v>440</v>
       </c>
       <c r="P103" s="139" t="n">
-        <v>205</v>
+        <v>349.9999999999999</v>
       </c>
       <c r="Q103" s="145" t="n">
-        <v>0.576923076923077</v>
+        <v>0.7</v>
       </c>
       <c r="R103" s="157" t="inlineStr">
         <is>
@@ -11585,10 +11585,10 @@
         <v>470</v>
       </c>
       <c r="P104" s="139" t="n">
-        <v>300</v>
+        <v>300.2727272727273</v>
       </c>
       <c r="Q104" s="145" t="n">
-        <v>0.56948275862069</v>
+        <v>0.5694827586206896</v>
       </c>
       <c r="R104" s="157" t="inlineStr">
         <is>
@@ -11644,10 +11644,10 @@
         <v>48</v>
       </c>
       <c r="K105" s="168" t="n">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="L105" s="168" t="n">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="M105" s="168" t="n">
         <v>2980</v>
@@ -11659,10 +11659,10 @@
         <v>1990</v>
       </c>
       <c r="P105" s="148" t="n">
-        <v>1212</v>
+        <v>1208</v>
       </c>
       <c r="Q105" s="145" t="n">
-        <v>0.550909090909091</v>
+        <v>0.5490909090909091</v>
       </c>
       <c r="R105" s="167" t="inlineStr">
         <is>
@@ -11792,10 +11792,10 @@
         <v>51</v>
       </c>
       <c r="K107" s="168" t="n">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="L107" s="168" t="n">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="M107" s="168" t="n">
         <v>3530</v>
@@ -11807,10 +11807,10 @@
         <v>2370</v>
       </c>
       <c r="P107" s="148" t="n">
-        <v>1465</v>
+        <v>1464.090909090909</v>
       </c>
       <c r="Q107" s="145" t="n">
-        <v>0.561533101045296</v>
+        <v>0.5611498257839721</v>
       </c>
       <c r="R107" s="167" t="inlineStr">
         <is>
@@ -11872,19 +11872,19 @@
         <v>102</v>
       </c>
       <c r="M108" s="158" t="n">
-        <v>330</v>
+        <v>540</v>
       </c>
       <c r="N108" s="158" t="n">
-        <v>280</v>
+        <v>460</v>
       </c>
       <c r="O108" s="158" t="n">
-        <v>230</v>
+        <v>380</v>
       </c>
       <c r="P108" s="139" t="n">
-        <v>153</v>
+        <v>316.1818181818181</v>
       </c>
       <c r="Q108" s="145" t="n">
-        <v>0.599285714285714</v>
+        <v>0.7560869565217391</v>
       </c>
       <c r="R108" s="157" t="inlineStr">
         <is>
@@ -11940,25 +11940,25 @@
         <v>0</v>
       </c>
       <c r="K109" s="158" t="n">
-        <v>100</v>
+        <v>100.5</v>
       </c>
       <c r="L109" s="158" t="n">
-        <v>132</v>
+        <v>132.5</v>
       </c>
       <c r="M109" s="158" t="n">
+        <v>650</v>
+      </c>
+      <c r="N109" s="158" t="n">
+        <v>510</v>
+      </c>
+      <c r="O109" s="158" t="n">
         <v>420</v>
       </c>
-      <c r="N109" s="158" t="n">
-        <v>330</v>
-      </c>
-      <c r="O109" s="158" t="n">
-        <v>270</v>
-      </c>
       <c r="P109" s="139" t="n">
-        <v>168</v>
+        <v>331.1363636363636</v>
       </c>
       <c r="Q109" s="145" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.7142156862745098</v>
       </c>
       <c r="R109" s="157" t="inlineStr">
         <is>
@@ -12020,19 +12020,19 @@
         <v>105</v>
       </c>
       <c r="M110" s="158" t="n">
-        <v>330</v>
+        <v>540</v>
       </c>
       <c r="N110" s="158" t="n">
-        <v>280</v>
+        <v>460</v>
       </c>
       <c r="O110" s="158" t="n">
-        <v>230</v>
+        <v>380</v>
       </c>
       <c r="P110" s="139" t="n">
-        <v>150</v>
+        <v>313.1818181818181</v>
       </c>
       <c r="Q110" s="145" t="n">
-        <v>0.5875</v>
+        <v>0.7489130434782608</v>
       </c>
       <c r="R110" s="157" t="inlineStr">
         <is>
@@ -12094,19 +12094,19 @@
         <v>105</v>
       </c>
       <c r="M111" s="158" t="n">
-        <v>360</v>
+        <v>570</v>
       </c>
       <c r="N111" s="158" t="n">
-        <v>290</v>
+        <v>460</v>
       </c>
       <c r="O111" s="158" t="n">
-        <v>240</v>
+        <v>380</v>
       </c>
       <c r="P111" s="139" t="n">
-        <v>159</v>
+        <v>313.1818181818181</v>
       </c>
       <c r="Q111" s="145" t="n">
-        <v>0.601724137931035</v>
+        <v>0.7489130434782608</v>
       </c>
       <c r="R111" s="157" t="inlineStr">
         <is>
@@ -12168,19 +12168,19 @@
         <v>55</v>
       </c>
       <c r="M112" s="158" t="n">
-        <v>200</v>
+        <v>420</v>
       </c>
       <c r="N112" s="158" t="n">
-        <v>170</v>
+        <v>360</v>
       </c>
       <c r="O112" s="158" t="n">
-        <v>140</v>
+        <v>300</v>
       </c>
       <c r="P112" s="139" t="n">
-        <v>100</v>
+        <v>272.2727272727273</v>
       </c>
       <c r="Q112" s="145" t="n">
-        <v>0.644117647058824</v>
+        <v>0.8319444444444445</v>
       </c>
       <c r="R112" s="157" t="inlineStr">
         <is>
@@ -12251,10 +12251,10 @@
         <v>360</v>
       </c>
       <c r="P113" s="179" t="n">
-        <v>249</v>
+        <v>249.0909090909091</v>
       </c>
       <c r="Q113" s="174" t="n">
-        <v>0.608888888888889</v>
+        <v>0.6088888888888888</v>
       </c>
       <c r="R113" s="157" t="inlineStr">
         <is>
@@ -12316,19 +12316,19 @@
         <v>90</v>
       </c>
       <c r="M114" s="158" t="n">
-        <v>310</v>
+        <v>530</v>
       </c>
       <c r="N114" s="158" t="n">
-        <v>250</v>
+        <v>430</v>
       </c>
       <c r="O114" s="158" t="n">
-        <v>200</v>
+        <v>340</v>
       </c>
       <c r="P114" s="139" t="n">
-        <v>137</v>
+        <v>300.9090909090909</v>
       </c>
       <c r="Q114" s="145" t="n">
-        <v>0.604</v>
+        <v>0.7697674418604651</v>
       </c>
       <c r="R114" s="157" t="inlineStr">
         <is>
@@ -12399,10 +12399,10 @@
         <v>470</v>
       </c>
       <c r="P115" s="139" t="n">
-        <v>317</v>
+        <v>317.2727272727273</v>
       </c>
       <c r="Q115" s="145" t="n">
-        <v>0.601724137931035</v>
+        <v>0.6017241379310345</v>
       </c>
       <c r="R115" s="157" t="inlineStr">
         <is>
@@ -12473,10 +12473,10 @@
         <v>420</v>
       </c>
       <c r="P116" s="139" t="n">
-        <v>284</v>
+        <v>283.8181818181818</v>
       </c>
       <c r="Q116" s="145" t="n">
-        <v>0.589056603773585</v>
+        <v>0.5890566037735848</v>
       </c>
       <c r="R116" s="157" t="inlineStr">
         <is>
@@ -12533,10 +12533,10 @@
         <v>30</v>
       </c>
       <c r="K117" s="144" t="n">
-        <v>220</v>
+        <v>220.5</v>
       </c>
       <c r="L117" s="144" t="n">
-        <v>302</v>
+        <v>302.5</v>
       </c>
       <c r="M117" s="144" t="n">
         <v>1000</v>
@@ -12548,10 +12548,10 @@
         <v>640</v>
       </c>
       <c r="P117" s="147" t="n">
-        <v>425</v>
+        <v>424.7727272727273</v>
       </c>
       <c r="Q117" s="145" t="n">
-        <v>0.58475</v>
+        <v>0.5840625</v>
       </c>
       <c r="R117" s="143" t="inlineStr">
         <is>
@@ -12622,10 +12622,10 @@
         <v>860</v>
       </c>
       <c r="P118" s="147" t="n">
-        <v>545</v>
+        <v>544.5454545454545</v>
       </c>
       <c r="Q118" s="145" t="n">
-        <v>0.570476190476191</v>
+        <v>0.5704761904761905</v>
       </c>
       <c r="R118" s="143" t="inlineStr">
         <is>
@@ -12682,10 +12682,10 @@
         <v>30</v>
       </c>
       <c r="K119" s="144" t="n">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="L119" s="144" t="n">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="M119" s="144" t="n">
         <v>1100</v>
@@ -12697,10 +12697,10 @@
         <v>720</v>
       </c>
       <c r="P119" s="147" t="n">
-        <v>474</v>
+        <v>476.090909090909</v>
       </c>
       <c r="Q119" s="145" t="n">
-        <v>0.5859550561797749</v>
+        <v>0.5884269662921348</v>
       </c>
       <c r="R119" s="143" t="inlineStr">
         <is>
@@ -12757,10 +12757,10 @@
         <v>55</v>
       </c>
       <c r="K120" s="151" t="n">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="L120" s="151" t="n">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="M120" s="151" t="n">
         <v>3530</v>
@@ -12772,10 +12772,10 @@
         <v>2310</v>
       </c>
       <c r="P120" s="162" t="n">
-        <v>1604</v>
+        <v>1608.090909090909</v>
       </c>
       <c r="Q120" s="145" t="n">
-        <v>0.614808362369338</v>
+        <v>0.6163414634146341</v>
       </c>
       <c r="R120" s="150" t="inlineStr">
         <is>
@@ -12847,10 +12847,10 @@
         <v>2920</v>
       </c>
       <c r="P121" s="162" t="n">
-        <v>1929</v>
+        <v>1929.090909090909</v>
       </c>
       <c r="Q121" s="145" t="n">
-        <v>0.601133144475921</v>
+        <v>0.6011331444759207</v>
       </c>
       <c r="R121" s="150" t="inlineStr">
         <is>
@@ -12907,10 +12907,10 @@
         <v>30</v>
       </c>
       <c r="K122" s="151" t="n">
-        <v>300</v>
+        <v>252</v>
       </c>
       <c r="L122" s="151" t="n">
-        <v>425</v>
+        <v>377</v>
       </c>
       <c r="M122" s="151" t="n">
         <v>1300</v>
@@ -12922,10 +12922,10 @@
         <v>840</v>
       </c>
       <c r="P122" s="162" t="n">
-        <v>539</v>
+        <v>568.4545454545454</v>
       </c>
       <c r="Q122" s="145" t="n">
-        <v>0.57</v>
+        <v>0.60125</v>
       </c>
       <c r="R122" s="150" t="inlineStr">
         <is>
@@ -12981,10 +12981,10 @@
         <v>35</v>
       </c>
       <c r="K123" s="151" t="n">
-        <v>410</v>
+        <v>360</v>
       </c>
       <c r="L123" s="151" t="n">
-        <v>580</v>
+        <v>530</v>
       </c>
       <c r="M123" s="151" t="n">
         <v>1770</v>
@@ -12996,10 +12996,10 @@
         <v>1150</v>
       </c>
       <c r="P123" s="162" t="n">
-        <v>702</v>
+        <v>751.8181818181818</v>
       </c>
       <c r="Q123" s="145" t="n">
-        <v>0.547</v>
+        <v>0.5865248226950355</v>
       </c>
       <c r="R123" s="150" t="inlineStr">
         <is>
@@ -13056,10 +13056,10 @@
         <v>30</v>
       </c>
       <c r="K124" s="151" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="L124" s="151" t="n">
-        <v>515</v>
+        <v>465</v>
       </c>
       <c r="M124" s="151" t="n">
         <v>1550</v>
@@ -13071,10 +13071,10 @@
         <v>1010</v>
       </c>
       <c r="P124" s="162" t="n">
-        <v>612</v>
+        <v>662.2727272727273</v>
       </c>
       <c r="Q124" s="145" t="n">
-        <v>0.543</v>
+        <v>0.5875</v>
       </c>
       <c r="R124" s="150" t="inlineStr">
         <is>
@@ -13131,10 +13131,10 @@
         <v>55</v>
       </c>
       <c r="K125" s="151" t="n">
-        <v>1055</v>
+        <v>1005</v>
       </c>
       <c r="L125" s="151" t="n">
-        <v>1410</v>
+        <v>1360</v>
       </c>
       <c r="M125" s="151" t="n">
         <v>4640</v>
@@ -13146,10 +13146,10 @@
         <v>3020</v>
       </c>
       <c r="P125" s="162" t="n">
-        <v>1954</v>
+        <v>2003.636363636364</v>
       </c>
       <c r="Q125" s="145" t="n">
-        <v>0.581</v>
+        <v>0.5956756756756757</v>
       </c>
       <c r="R125" s="150" t="inlineStr">
         <is>
@@ -13206,10 +13206,10 @@
         <v>65</v>
       </c>
       <c r="K126" s="151" t="n">
-        <v>1292</v>
+        <v>1242</v>
       </c>
       <c r="L126" s="151" t="n">
-        <v>1742</v>
+        <v>1692</v>
       </c>
       <c r="M126" s="151" t="n">
         <v>5720</v>
@@ -13221,10 +13221,10 @@
         <v>3720</v>
       </c>
       <c r="P126" s="162" t="n">
-        <v>2403</v>
+        <v>2453.454545454545</v>
       </c>
       <c r="Q126" s="145" t="n">
-        <v>0.58</v>
+        <v>0.5918421052631578</v>
       </c>
       <c r="R126" s="150" t="inlineStr">
         <is>
@@ -13280,25 +13280,25 @@
         <v>0</v>
       </c>
       <c r="K127" s="158" t="n">
-        <v>100</v>
+        <v>100.5</v>
       </c>
       <c r="L127" s="158" t="n">
-        <v>135</v>
+        <v>135.5</v>
       </c>
       <c r="M127" s="158" t="n">
-        <v>470</v>
+        <v>640</v>
       </c>
       <c r="N127" s="158" t="n">
-        <v>380</v>
+        <v>520</v>
       </c>
       <c r="O127" s="158" t="n">
-        <v>300</v>
+        <v>410</v>
       </c>
       <c r="P127" s="139" t="n">
-        <v>210</v>
+        <v>337.2272727272727</v>
       </c>
       <c r="Q127" s="145" t="n">
-        <v>0.609210526315789</v>
+        <v>0.7133653846153846</v>
       </c>
       <c r="R127" s="157" t="inlineStr">
         <is>
@@ -13369,10 +13369,10 @@
         <v>2370</v>
       </c>
       <c r="P128" s="162" t="n">
-        <v>1544</v>
+        <v>1544.090909090909</v>
       </c>
       <c r="Q128" s="145" t="n">
-        <v>0.5918118466898959</v>
+        <v>0.5918118466898955</v>
       </c>
       <c r="R128" s="167" t="inlineStr">
         <is>
@@ -13428,25 +13428,25 @@
         <v>0</v>
       </c>
       <c r="K129" s="158" t="n">
-        <v>100</v>
+        <v>100.5</v>
       </c>
       <c r="L129" s="158" t="n">
-        <v>125</v>
+        <v>125.5</v>
       </c>
       <c r="M129" s="158" t="n">
-        <v>420</v>
+        <v>640</v>
       </c>
       <c r="N129" s="158" t="n">
-        <v>330</v>
+        <v>500</v>
       </c>
       <c r="O129" s="158" t="n">
-        <v>270</v>
+        <v>410</v>
       </c>
       <c r="P129" s="139" t="n">
-        <v>175</v>
+        <v>329.0454545454545</v>
       </c>
       <c r="Q129" s="145" t="n">
-        <v>0.583333333333333</v>
+        <v>0.7239</v>
       </c>
       <c r="R129" s="157" t="inlineStr">
         <is>
@@ -13509,19 +13509,19 @@
         <v>115</v>
       </c>
       <c r="M130" s="138" t="n">
+        <v>600</v>
+      </c>
+      <c r="N130" s="138" t="n">
+        <v>480</v>
+      </c>
+      <c r="O130" s="138" t="n">
         <v>390</v>
       </c>
-      <c r="N130" s="138" t="n">
-        <v>310</v>
-      </c>
-      <c r="O130" s="138" t="n">
-        <v>250</v>
-      </c>
       <c r="P130" s="139" t="n">
-        <v>167</v>
+        <v>321.3636363636363</v>
       </c>
       <c r="Q130" s="145" t="n">
-        <v>0.5919354838709679</v>
+        <v>0.7364583333333333</v>
       </c>
       <c r="R130" s="137" t="inlineStr">
         <is>
@@ -13593,7 +13593,7 @@
         <v>400</v>
       </c>
       <c r="P131" s="139" t="n">
-        <v>265</v>
+        <v>264.5454545454545</v>
       </c>
       <c r="Q131" s="145" t="n">
         <v>0.582</v>
@@ -13659,19 +13659,19 @@
         <v>82</v>
       </c>
       <c r="M132" s="144" t="n">
-        <v>300</v>
+        <v>520</v>
       </c>
       <c r="N132" s="144" t="n">
-        <v>240</v>
+        <v>420</v>
       </c>
       <c r="O132" s="144" t="n">
-        <v>190</v>
+        <v>330</v>
       </c>
       <c r="P132" s="139" t="n">
-        <v>136</v>
+        <v>299.8181818181818</v>
       </c>
       <c r="Q132" s="145" t="n">
-        <v>0.624166666666667</v>
+        <v>0.7852380952380953</v>
       </c>
       <c r="R132" s="143" t="inlineStr">
         <is>
@@ -13733,19 +13733,19 @@
         <v>167</v>
       </c>
       <c r="M133" s="144" t="n">
-        <v>530</v>
+        <v>730</v>
       </c>
       <c r="N133" s="144" t="n">
-        <v>420</v>
+        <v>580</v>
       </c>
       <c r="O133" s="144" t="n">
-        <v>350</v>
+        <v>480</v>
       </c>
       <c r="P133" s="139" t="n">
-        <v>215</v>
+        <v>360.2727272727273</v>
       </c>
       <c r="Q133" s="145" t="n">
-        <v>0.562619047619048</v>
+        <v>0.6832758620689655</v>
       </c>
       <c r="R133" s="143" t="inlineStr">
         <is>
@@ -13801,25 +13801,25 @@
         <v>0</v>
       </c>
       <c r="K134" s="158" t="n">
-        <v>100</v>
+        <v>100.5</v>
       </c>
       <c r="L134" s="158" t="n">
-        <v>130</v>
+        <v>130.5</v>
       </c>
       <c r="M134" s="158" t="n">
-        <v>450</v>
+        <v>640</v>
       </c>
       <c r="N134" s="158" t="n">
-        <v>360</v>
+        <v>510</v>
       </c>
       <c r="O134" s="158" t="n">
-        <v>280</v>
+        <v>400</v>
       </c>
       <c r="P134" s="139" t="n">
-        <v>197</v>
+        <v>333.1363636363636</v>
       </c>
       <c r="Q134" s="145" t="n">
-        <v>0.602777777777778</v>
+        <v>0.7185294117647059</v>
       </c>
       <c r="R134" s="157" t="inlineStr">
         <is>
@@ -13882,19 +13882,19 @@
         <v>215</v>
       </c>
       <c r="M135" s="158" t="n">
-        <v>660</v>
+        <v>850</v>
       </c>
       <c r="N135" s="158" t="n">
-        <v>530</v>
+        <v>680</v>
       </c>
       <c r="O135" s="158" t="n">
-        <v>420</v>
+        <v>540</v>
       </c>
       <c r="P135" s="139" t="n">
-        <v>267</v>
+        <v>403.1818181818181</v>
       </c>
       <c r="Q135" s="145" t="n">
-        <v>0.55377358490566</v>
+        <v>0.6522058823529412</v>
       </c>
       <c r="R135" s="157" t="inlineStr">
         <is>
@@ -13950,25 +13950,25 @@
         <v>0</v>
       </c>
       <c r="K136" s="158" t="n">
-        <v>100</v>
+        <v>100.5</v>
       </c>
       <c r="L136" s="158" t="n">
-        <v>120</v>
+        <v>120.5</v>
       </c>
       <c r="M136" s="158" t="n">
-        <v>420</v>
+        <v>620</v>
       </c>
       <c r="N136" s="158" t="n">
-        <v>330</v>
+        <v>490</v>
       </c>
       <c r="O136" s="158" t="n">
-        <v>270</v>
+        <v>400</v>
       </c>
       <c r="P136" s="139" t="n">
-        <v>180</v>
+        <v>324.9545454545454</v>
       </c>
       <c r="Q136" s="145" t="n">
-        <v>0.6</v>
+        <v>0.7294897959183674</v>
       </c>
       <c r="R136" s="157" t="inlineStr">
         <is>
@@ -14039,7 +14039,7 @@
         <v>400</v>
       </c>
       <c r="P137" s="139" t="n">
-        <v>265</v>
+        <v>264.5454545454545</v>
       </c>
       <c r="Q137" s="145" t="n">
         <v>0.582</v>
@@ -14099,10 +14099,10 @@
         <v>0</v>
       </c>
       <c r="K138" s="183" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L138" s="183" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="M138" s="183" t="n">
         <v>940</v>
@@ -14114,10 +14114,10 @@
         <v>610</v>
       </c>
       <c r="P138" s="147" t="n">
-        <v>402</v>
+        <v>400.8181818181818</v>
       </c>
       <c r="Q138" s="145" t="n">
-        <v>0.589333333333333</v>
+        <v>0.5878666666666666</v>
       </c>
       <c r="R138" s="182" t="inlineStr">
         <is>
@@ -14189,10 +14189,10 @@
         <v>940</v>
       </c>
       <c r="P139" s="147" t="n">
-        <v>615</v>
+        <v>614.5454545454545</v>
       </c>
       <c r="Q139" s="145" t="n">
-        <v>0.582758620689655</v>
+        <v>0.5827586206896551</v>
       </c>
       <c r="R139" s="182" t="inlineStr">
         <is>
@@ -14254,19 +14254,19 @@
         <v>150</v>
       </c>
       <c r="M140" s="186" t="n">
-        <v>500</v>
+        <v>690</v>
       </c>
       <c r="N140" s="186" t="n">
-        <v>400</v>
+        <v>550</v>
       </c>
       <c r="O140" s="186" t="n">
-        <v>320</v>
+        <v>440</v>
       </c>
       <c r="P140" s="139" t="n">
-        <v>214</v>
+        <v>349.9999999999999</v>
       </c>
       <c r="Q140" s="145" t="n">
-        <v>0.5875</v>
+        <v>0.7</v>
       </c>
       <c r="R140" s="185" t="inlineStr">
         <is>
@@ -14328,19 +14328,19 @@
         <v>115</v>
       </c>
       <c r="M141" s="186" t="n">
+        <v>600</v>
+      </c>
+      <c r="N141" s="186" t="n">
+        <v>480</v>
+      </c>
+      <c r="O141" s="186" t="n">
         <v>390</v>
       </c>
-      <c r="N141" s="186" t="n">
-        <v>310</v>
-      </c>
-      <c r="O141" s="186" t="n">
-        <v>250</v>
-      </c>
       <c r="P141" s="139" t="n">
-        <v>167</v>
+        <v>321.3636363636363</v>
       </c>
       <c r="Q141" s="145" t="n">
-        <v>0.5919354838709679</v>
+        <v>0.7364583333333333</v>
       </c>
       <c r="R141" s="185" t="inlineStr">
         <is>
@@ -14396,10 +14396,10 @@
         <v>0</v>
       </c>
       <c r="K142" s="154" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L142" s="154" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M142" s="154" t="n">
         <v>940</v>
@@ -14411,10 +14411,10 @@
         <v>610</v>
       </c>
       <c r="P142" s="139" t="n">
-        <v>387</v>
+        <v>385.8181818181818</v>
       </c>
       <c r="Q142" s="145" t="n">
-        <v>0.567333333333333</v>
+        <v>0.5658666666666666</v>
       </c>
       <c r="R142" s="153" t="inlineStr">
         <is>
@@ -14471,10 +14471,10 @@
         <v>0</v>
       </c>
       <c r="K143" s="154" t="n">
-        <v>300</v>
+        <v>301.5</v>
       </c>
       <c r="L143" s="154" t="n">
-        <v>430</v>
+        <v>431.5</v>
       </c>
       <c r="M143" s="154" t="n">
         <v>1380</v>
@@ -14486,10 +14486,10 @@
         <v>890</v>
       </c>
       <c r="P143" s="147" t="n">
-        <v>570</v>
+        <v>568.4999999999999</v>
       </c>
       <c r="Q143" s="145" t="n">
-        <v>0.57</v>
+        <v>0.5685</v>
       </c>
       <c r="R143" s="153" t="inlineStr">
         <is>
@@ -14563,7 +14563,7 @@
         <v>680</v>
       </c>
       <c r="Q144" s="145" t="n">
-        <v>0.566666666666667</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="R144" s="153" t="inlineStr">
         <is>
@@ -14575,6 +14575,7 @@
         <v>68</v>
       </c>
     </row>
+    <row r="145"/>
     <row r="146">
       <c r="A146" s="101" t="inlineStr">
         <is>

</xml_diff>